<commit_message>
added rules in different languages
</commit_message>
<xml_diff>
--- a/cbom_rules_reference.xlsx
+++ b/cbom_rules_reference.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30002"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="4" documentId="11_2C93AB4C4C85AFB228BD8BE0D0714A6BD02A75E1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D984BD36-D580-445E-ADE1-FD4702073F5A}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CERT-In Rules" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,23 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'CERT-In Rules'!$A$1:$C$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Other Standards Rules'!$A$1:$C$1</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -412,7 +428,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -825,14 +841,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C31"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="21.81640625" customWidth="1"/>
+    <col min="1" max="1" width="21.85546875" customWidth="1"/>
     <col min="2" max="2" width="46" customWidth="1"/>
     <col min="3" max="3" width="62" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="27.95" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -843,7 +859,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="21.95" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -854,7 +870,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="21.95" customHeight="1">
       <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
@@ -865,7 +881,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="21.95" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
@@ -876,7 +892,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="21.95" customHeight="1">
       <c r="A5" s="4" t="s">
         <v>11</v>
       </c>
@@ -887,7 +903,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="21.95" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
@@ -898,7 +914,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="21.95" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>15</v>
       </c>
@@ -909,7 +925,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="21.95" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>17</v>
       </c>
@@ -920,7 +936,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="21.95" customHeight="1">
       <c r="A9" s="4" t="s">
         <v>19</v>
       </c>
@@ -931,7 +947,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" ht="21.95" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>21</v>
       </c>
@@ -942,7 +958,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" ht="21.95" customHeight="1">
       <c r="A11" s="4" t="s">
         <v>23</v>
       </c>
@@ -953,7 +969,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="21.95" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>26</v>
       </c>
@@ -964,7 +980,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="21.95" customHeight="1">
       <c r="A13" s="4" t="s">
         <v>29</v>
       </c>
@@ -975,7 +991,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="21.95" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>32</v>
       </c>
@@ -986,7 +1002,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="21.95" customHeight="1">
       <c r="A15" s="4" t="s">
         <v>34</v>
       </c>
@@ -997,7 +1013,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="21.95" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>36</v>
       </c>
@@ -1008,7 +1024,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" ht="21.95" customHeight="1">
       <c r="A17" s="4" t="s">
         <v>38</v>
       </c>
@@ -1019,7 +1035,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" ht="21.95" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>41</v>
       </c>
@@ -1030,7 +1046,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" ht="21.95" customHeight="1">
       <c r="A19" s="4" t="s">
         <v>43</v>
       </c>
@@ -1041,7 +1057,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" ht="21.95" customHeight="1">
       <c r="A20" s="2" t="s">
         <v>45</v>
       </c>
@@ -1052,7 +1068,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" ht="21.95" customHeight="1">
       <c r="A21" s="4" t="s">
         <v>47</v>
       </c>
@@ -1063,7 +1079,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" ht="21.95" customHeight="1">
       <c r="A22" s="2" t="s">
         <v>49</v>
       </c>
@@ -1074,7 +1090,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" ht="21.95" customHeight="1">
       <c r="A23" s="4" t="s">
         <v>51</v>
       </c>
@@ -1085,7 +1101,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" ht="21.95" customHeight="1">
       <c r="A24" s="2" t="s">
         <v>54</v>
       </c>
@@ -1096,7 +1112,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" ht="21.95" customHeight="1">
       <c r="A25" s="4" t="s">
         <v>57</v>
       </c>
@@ -1107,7 +1123,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" ht="21.95" customHeight="1">
       <c r="A26" s="2" t="s">
         <v>59</v>
       </c>
@@ -1118,7 +1134,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" ht="21.95" customHeight="1">
       <c r="A27" s="4" t="s">
         <v>61</v>
       </c>
@@ -1129,7 +1145,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" ht="21.95" customHeight="1">
       <c r="A28" s="2" t="s">
         <v>64</v>
       </c>
@@ -1140,7 +1156,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" ht="21.95" customHeight="1">
       <c r="A29" s="4" t="s">
         <v>66</v>
       </c>
@@ -1151,7 +1167,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" ht="21.95" customHeight="1">
       <c r="A30" s="2" t="s">
         <v>69</v>
       </c>
@@ -1162,7 +1178,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" ht="21.95" customHeight="1">
       <c r="A31" s="4" t="s">
         <v>71</v>
       </c>
@@ -1183,14 +1199,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="21.7265625" customWidth="1"/>
+    <col min="1" max="1" width="21.7109375" customWidth="1"/>
     <col min="2" max="2" width="56" customWidth="1"/>
     <col min="3" max="3" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="27.95" customHeight="1">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1201,7 +1217,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="21.95" customHeight="1">
       <c r="A2" s="7" t="s">
         <v>75</v>
       </c>
@@ -1212,7 +1228,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="21.95" customHeight="1">
       <c r="A3" s="4" t="s">
         <v>78</v>
       </c>
@@ -1223,7 +1239,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="21.95" customHeight="1">
       <c r="A4" s="7" t="s">
         <v>81</v>
       </c>
@@ -1234,7 +1250,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="21.95" customHeight="1">
       <c r="A5" s="4" t="s">
         <v>84</v>
       </c>
@@ -1245,7 +1261,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="21.95" customHeight="1">
       <c r="A6" s="7" t="s">
         <v>86</v>
       </c>
@@ -1256,7 +1272,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="21.95" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>89</v>
       </c>
@@ -1267,7 +1283,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="21.95" customHeight="1">
       <c r="A8" s="7" t="s">
         <v>92</v>
       </c>
@@ -1278,7 +1294,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="21.95" customHeight="1">
       <c r="A9" s="4" t="s">
         <v>94</v>
       </c>
@@ -1289,7 +1305,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" ht="21.95" customHeight="1">
       <c r="A10" s="7" t="s">
         <v>96</v>
       </c>
@@ -1300,7 +1316,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" ht="21.95" customHeight="1">
       <c r="A11" s="4" t="s">
         <v>98</v>
       </c>
@@ -1311,7 +1327,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="21.95" customHeight="1">
       <c r="A12" s="7" t="s">
         <v>100</v>
       </c>
@@ -1322,7 +1338,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="21.95" customHeight="1">
       <c r="A13" s="4" t="s">
         <v>103</v>
       </c>
@@ -1333,7 +1349,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="21.95" customHeight="1">
       <c r="A14" s="7" t="s">
         <v>106</v>
       </c>
@@ -1344,7 +1360,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="21.95" customHeight="1">
       <c r="A15" s="4" t="s">
         <v>109</v>
       </c>
@@ -1355,7 +1371,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="21.95" customHeight="1">
       <c r="A16" s="7" t="s">
         <v>112</v>
       </c>
@@ -1366,7 +1382,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" ht="21.95" customHeight="1">
       <c r="A17" s="4" t="s">
         <v>115</v>
       </c>
@@ -1377,7 +1393,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" ht="21.95" customHeight="1">
       <c r="A18" s="7" t="s">
         <v>118</v>
       </c>
@@ -1388,7 +1404,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" ht="21.95" customHeight="1">
       <c r="A19" s="4" t="s">
         <v>121</v>
       </c>
@@ -1399,7 +1415,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" ht="21.95" customHeight="1">
       <c r="A20" s="7" t="s">
         <v>124</v>
       </c>

</xml_diff>